<commit_message>
tx-export-convert Fix sorting, commission for FX. Add DIV support
USD dividends will now add to your USD.FX amount.
</commit_message>
<xml_diff>
--- a/test/QT_Test_Export.xlsx
+++ b/test/QT_Test_Export.xlsx
@@ -5,13 +5,14 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="TXs" sheetId="1" state="visible" r:id="rId2"/>
     <sheet name="FXTs" sheetId="2" state="visible" r:id="rId3"/>
     <sheet name="TX Errors" sheetId="3" state="visible" r:id="rId4"/>
     <sheet name="FXT Errors" sheetId="4" state="visible" r:id="rId5"/>
+    <sheet name="Sorting" sheetId="5" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
@@ -23,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="146">
   <si>
     <t xml:space="preserve">Transaction Date</t>
   </si>
@@ -245,6 +246,9 @@
   </si>
   <si>
     <t xml:space="preserve">DIV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30.5</t>
   </si>
   <si>
     <t xml:space="preserve">Ignored actions</t>
@@ -557,7 +561,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:O26"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.92"/>
@@ -1226,27 +1230,58 @@
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0"/>
-      <c r="B15" s="0"/>
-      <c r="C15" s="0"/>
-      <c r="D15" s="0"/>
-      <c r="E15" s="0"/>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0"/>
-      <c r="K15" s="0"/>
-      <c r="L15" s="0"/>
-      <c r="M15" s="0"/>
-      <c r="N15" s="0"/>
-      <c r="O15" s="0"/>
-      <c r="P15" s="0"/>
+      <c r="A15" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L15" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1"/>
+      <c r="A17" s="1" t="s">
+        <v>69</v>
+      </c>
       <c r="B17" s="1" t="s">
-        <v>19</v>
+        <v>70</v>
       </c>
       <c r="C17" s="0" t="s">
         <v>73</v>
@@ -1283,63 +1318,67 @@
         <v>19</v>
       </c>
       <c r="O17" s="0" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="1"/>
+        <v>69</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>70</v>
+      </c>
       <c r="C18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O18" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="B19" s="1"/>
       <c r="C19" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D19" s="1"/>
+      <c r="D19" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="E19" s="1" t="s">
         <v>19</v>
       </c>
@@ -1361,15 +1400,15 @@
       <c r="K19" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="L19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="N19" s="1" t="s">
         <v>19</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1382,10 +1421,10 @@
       <c r="C20" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="F20" s="1" t="s">
         <v>19</v>
       </c>
@@ -1407,12 +1446,12 @@
       <c r="L20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="O20" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1428,10 +1467,10 @@
       <c r="D21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="G21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1453,11 +1492,9 @@
       <c r="M21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N21" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="N21" s="1"/>
       <c r="O21" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1476,10 +1513,10 @@
       <c r="E22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="H22" s="1" t="s">
         <v>19</v>
       </c>
@@ -1502,7 +1539,7 @@
         <v>19</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1524,10 +1561,10 @@
       <c r="F23" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="I23" s="1" t="s">
         <v>19</v>
       </c>
@@ -1547,7 +1584,7 @@
         <v>19</v>
       </c>
       <c r="O23" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1572,10 +1609,10 @@
       <c r="G24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H24" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="J24" s="1" t="s">
         <v>19</v>
       </c>
@@ -1592,7 +1629,7 @@
         <v>19</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,7 +1639,9 @@
       <c r="B25" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C25" s="1"/>
+      <c r="C25" s="1" t="s">
+        <v>82</v>
+      </c>
       <c r="D25" s="1" t="s">
         <v>19</v>
       </c>
@@ -1618,10 +1657,10 @@
       <c r="H25" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I25" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="K25" s="1" t="s">
         <v>19</v>
       </c>
@@ -1635,7 +1674,50 @@
         <v>19</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>82</v>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N26" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1711,13 +1793,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>19</v>
@@ -1738,7 +1820,7 @@
         <v>19</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>23</v>
@@ -1753,19 +1835,19 @@
         <v>33</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>19</v>
@@ -1786,7 +1868,7 @@
         <v>19</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>38</v>
@@ -1801,19 +1883,19 @@
         <v>33</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="P3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>19</v>
@@ -1834,7 +1916,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>38</v>
@@ -1849,19 +1931,19 @@
         <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>19</v>
@@ -1882,7 +1964,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>23</v>
@@ -1897,7 +1979,7 @@
         <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P5" s="1"/>
     </row>
@@ -1979,13 +2061,13 @@
         <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>19</v>
@@ -2018,7 +2100,7 @@
         <v>33</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2030,7 +2112,7 @@
         <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>19</v>
@@ -2063,12 +2145,12 @@
         <v>33</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>32</v>
@@ -2077,7 +2159,7 @@
         <v>17</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>19</v>
@@ -2110,7 +2192,7 @@
         <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2121,7 +2203,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>19</v>
@@ -2154,7 +2236,7 @@
         <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2165,10 +2247,10 @@
         <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>19</v>
@@ -2201,7 +2283,7 @@
         <v>24</v>
       </c>
       <c r="O6" s="0" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2246,7 +2328,7 @@
         <v>24</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2260,13 +2342,13 @@
         <v>17</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>21</v>
@@ -2293,7 +2375,7 @@
         <v>24</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2324,7 +2406,7 @@
         <v>51</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>19</v>
@@ -2354,7 +2436,7 @@
         <v>24</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2368,7 +2450,7 @@
         <v>17</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>19</v>
@@ -2398,7 +2480,7 @@
         <v>24</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2412,13 +2494,13 @@
         <v>51</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>21</v>
@@ -2445,7 +2527,7 @@
         <v>24</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2459,13 +2541,13 @@
         <v>17</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>21</v>
@@ -2492,7 +2574,7 @@
         <v>24</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2506,7 +2588,7 @@
         <v>51</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>19</v>
@@ -2536,7 +2618,7 @@
         <v>24</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2550,7 +2632,7 @@
         <v>17</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>19</v>
@@ -2580,7 +2662,7 @@
         <v>24</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2594,7 +2676,7 @@
         <v>51</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>19</v>
@@ -2603,7 +2685,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>19</v>
@@ -2627,7 +2709,7 @@
         <v>24</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2641,7 +2723,7 @@
         <v>17</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>19</v>
@@ -2650,7 +2732,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>19</v>
@@ -2674,7 +2756,7 @@
         <v>24</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="18" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2688,7 +2770,7 @@
         <v>51</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>19</v>
@@ -2718,7 +2800,7 @@
         <v>24</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2732,7 +2814,7 @@
         <v>17</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>19</v>
@@ -2762,7 +2844,7 @@
         <v>24</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2776,7 +2858,7 @@
         <v>51</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>19</v>
@@ -2791,7 +2873,7 @@
         <v>19</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>19</v>
@@ -2809,7 +2891,7 @@
         <v>24</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2823,7 +2905,7 @@
         <v>17</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>19</v>
@@ -2838,7 +2920,7 @@
         <v>19</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>19</v>
@@ -2856,7 +2938,7 @@
         <v>24</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3134,7 +3216,7 @@
         <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>19</v>
@@ -3167,18 +3249,18 @@
         <v>24</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>19</v>
@@ -3199,7 +3281,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>23</v>
@@ -3214,18 +3296,18 @@
         <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>19</v>
@@ -3246,7 +3328,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>38</v>
@@ -3261,18 +3343,18 @@
         <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>19</v>
@@ -3293,7 +3375,7 @@
         <v>19</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>23</v>
@@ -3308,18 +3390,18 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>19</v>
@@ -3340,7 +3422,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>38</v>
@@ -3355,18 +3437,18 @@
         <v>33</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>19</v>
@@ -3387,7 +3469,7 @@
         <v>19</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>23</v>
@@ -3402,18 +3484,18 @@
         <v>33</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>19</v>
@@ -3434,7 +3516,7 @@
         <v>19</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>23</v>
@@ -3449,18 +3531,18 @@
         <v>33</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="10" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>19</v>
@@ -3481,7 +3563,7 @@
         <v>19</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>38</v>
@@ -3496,18 +3578,18 @@
         <v>33</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="11" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>19</v>
@@ -3528,7 +3610,7 @@
         <v>19</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>38</v>
@@ -3543,18 +3625,18 @@
         <v>33</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>19</v>
@@ -3575,7 +3657,7 @@
         <v>19</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>23</v>
@@ -3590,18 +3672,18 @@
         <v>33</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>19</v>
@@ -3622,10 +3704,10 @@
         <v>19</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L13" s="1" t="n">
         <v>10000003</v>
@@ -3637,42 +3719,42 @@
         <v>33</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="K14" s="1" t="s">
         <v>133</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="K14" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="L14" s="1" t="n">
         <v>10000003</v>
@@ -3684,18 +3766,18 @@
         <v>33</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>19</v>
@@ -3716,7 +3798,7 @@
         <v>19</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>23</v>
@@ -3731,18 +3813,18 @@
         <v>33</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>19</v>
@@ -3763,7 +3845,7 @@
         <v>19</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>38</v>
@@ -3778,18 +3860,18 @@
         <v>33</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>19</v>
@@ -3810,10 +3892,10 @@
         <v>19</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L17" s="1" t="n">
         <v>10000003</v>
@@ -3825,18 +3907,18 @@
         <v>33</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="18" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>19</v>
@@ -3857,10 +3939,10 @@
         <v>19</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L18" s="1" t="n">
         <v>10000003</v>
@@ -3872,18 +3954,18 @@
         <v>33</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>19</v>
@@ -3904,7 +3986,7 @@
         <v>19</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>38</v>
@@ -3919,18 +4001,18 @@
         <v>33</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>19</v>
@@ -3951,10 +4033,10 @@
         <v>19</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L20" s="1" t="n">
         <v>10000003</v>
@@ -3966,18 +4048,18 @@
         <v>33</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>19</v>
@@ -3998,10 +4080,10 @@
         <v>19</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>10000003</v>
@@ -4013,18 +4095,18 @@
         <v>33</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>19</v>
@@ -4045,7 +4127,7 @@
         <v>19</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>23</v>
@@ -4060,7 +4142,7 @@
         <v>33</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4223,4 +4305,696 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:P25"/>
+  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="7.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="20.01"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" s="0" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="P2" s="1"/>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L3" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="P3" s="1"/>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L4" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="P4" s="1"/>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L5" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="P5" s="1"/>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L6" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I7" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O7" s="1"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I8" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L8" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N8" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O8" s="1"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I9" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N9" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O9" s="1"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I10" s="0" t="s">
+        <v>43</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L10" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O10" s="1"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+      <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+    </row>
+    <row r="14" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0"/>
+      <c r="B15" s="0"/>
+      <c r="C15" s="0"/>
+      <c r="D15" s="0"/>
+      <c r="E15" s="0"/>
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
+      <c r="K15" s="0"/>
+      <c r="L15" s="0"/>
+      <c r="M15" s="0"/>
+      <c r="N15" s="0"/>
+      <c r="O15" s="0"/>
+      <c r="P15" s="0"/>
+    </row>
+    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1"/>
+      <c r="B17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1"/>
+      <c r="B18" s="1"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="1"/>
+      <c r="O18" s="1"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1"/>
+      <c r="B19" s="1"/>
+      <c r="C19" s="1"/>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1"/>
+      <c r="H19" s="1"/>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="1"/>
+      <c r="O19" s="1"/>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1"/>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1"/>
+      <c r="H20" s="1"/>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+      <c r="K20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1"/>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1"/>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1"/>
+      <c r="O21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1"/>
+      <c r="B22" s="1"/>
+      <c r="C22" s="1"/>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1"/>
+      <c r="H22" s="1"/>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="1"/>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1"/>
+      <c r="B23" s="1"/>
+      <c r="C23" s="1"/>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="1"/>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1"/>
+      <c r="B24" s="1"/>
+      <c r="C24" s="1"/>
+      <c r="D24" s="1"/>
+      <c r="E24" s="1"/>
+      <c r="F24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1"/>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1"/>
+      <c r="B25" s="1"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add LIQ support to tx-export-convert
</commit_message>
<xml_diff>
--- a/test/QT_Test_Export.xlsx
+++ b/test/QT_Test_Export.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1084" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1096" uniqueCount="151">
   <si>
     <t xml:space="preserve">Transaction Date</t>
   </si>
@@ -167,6 +167,9 @@
     <t xml:space="preserve">2023-01-15 12:00:00 AM</t>
   </si>
   <si>
+    <t xml:space="preserve">BUY</t>
+  </si>
+  <si>
     <t xml:space="preserve">-1.00</t>
   </si>
   <si>
@@ -179,21 +182,24 @@
     <t xml:space="preserve">2023-01-17 12:00:00 AM</t>
   </si>
   <si>
+    <t xml:space="preserve">SELL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sell in TFSA (CAD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023-01-18 12:00:00 AM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2023-01-19 12:00:00 AM</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sell</t>
   </si>
   <si>
-    <t xml:space="preserve">1.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sell in TFSA (CAD)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-01-18 12:00:00 AM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2023-01-19 12:00:00 AM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sell in RRSP (CAD)</t>
   </si>
   <si>
@@ -245,10 +251,19 @@
     <t xml:space="preserve">DIS, behaves like buy</t>
   </si>
   <si>
+    <t xml:space="preserve">LIQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIQ, behaves like sell</t>
+  </si>
+  <si>
     <t xml:space="preserve">DIV</t>
   </si>
   <si>
     <t xml:space="preserve">30.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIV, behaves like buy of USD</t>
   </si>
   <si>
     <t xml:space="preserve">Ignored actions</t>
@@ -476,6 +491,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -561,8 +577,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:O26"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:O27"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.67"/>
@@ -861,7 +877,7 @@
         <v>46</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>42</v>
@@ -879,7 +895,7 @@
         <v>19</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>19</v>
@@ -897,18 +913,18 @@
         <v>33</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>18</v>
@@ -926,7 +942,7 @@
         <v>19</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>19</v>
@@ -944,18 +960,18 @@
         <v>24</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>18</v>
@@ -973,7 +989,7 @@
         <v>19</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>19</v>
@@ -991,18 +1007,18 @@
         <v>29</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>18</v>
@@ -1020,7 +1036,7 @@
         <v>19</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>19</v>
@@ -1038,18 +1054,18 @@
         <v>33</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>42</v>
@@ -1067,7 +1083,7 @@
         <v>19</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>19</v>
@@ -1085,18 +1101,18 @@
         <v>24</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>42</v>
@@ -1114,7 +1130,7 @@
         <v>19</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>19</v>
@@ -1132,18 +1148,18 @@
         <v>29</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>42</v>
@@ -1161,7 +1177,7 @@
         <v>19</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>19</v>
@@ -1179,18 +1195,18 @@
         <v>33</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>42</v>
@@ -1226,18 +1242,18 @@
         <v>33</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>42</v>
@@ -1245,20 +1261,20 @@
       <c r="E15" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>19</v>
+      <c r="F15" s="1" t="n">
+        <v>19</v>
+      </c>
+      <c r="G15" s="1" t="n">
+        <v>0</v>
       </c>
       <c r="H15" s="1" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>74</v>
+        <v>19</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>38</v>
@@ -1273,63 +1289,65 @@
         <v>33</v>
       </c>
       <c r="O15" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C17" s="0" t="s">
-        <v>73</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N17" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O17" s="0" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C16" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L16" s="1" t="n">
+        <v>10000003</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>77</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>19</v>
@@ -1352,55 +1370,57 @@
       <c r="J18" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="K18" s="1"/>
+      <c r="L18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O18" s="0" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K19" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="L18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O18" s="1" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L19" s="1"/>
+      <c r="L19" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="M19" s="1" t="s">
         <v>19</v>
       </c>
@@ -1408,20 +1428,20 @@
         <v>19</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="B20" s="1"/>
       <c r="C20" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D20" s="1"/>
+        <v>81</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="E20" s="1" t="s">
         <v>19</v>
       </c>
@@ -1443,15 +1463,15 @@
       <c r="K20" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="L20" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M20" s="1"/>
+      <c r="L20" s="1"/>
+      <c r="M20" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="N20" s="1" t="s">
         <v>19</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1462,12 +1482,12 @@
         <v>19</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="1"/>
+        <v>82</v>
+      </c>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="F21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1489,12 +1509,12 @@
       <c r="L21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="M21" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="O21" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1505,15 +1525,15 @@
         <v>19</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F22" s="1"/>
+      <c r="E22" s="1"/>
+      <c r="F22" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="G22" s="1" t="s">
         <v>19</v>
       </c>
@@ -1535,11 +1555,9 @@
       <c r="M22" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="N22" s="1" t="s">
-        <v>19</v>
-      </c>
+      <c r="N22" s="1"/>
       <c r="O22" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1550,41 +1568,41 @@
         <v>19</v>
       </c>
       <c r="C23" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="K23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O23" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="N23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="O23" s="1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1595,7 +1613,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>19</v>
@@ -1606,10 +1624,10 @@
       <c r="F24" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G24" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H24" s="1"/>
+      <c r="G24" s="1"/>
+      <c r="H24" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="I24" s="1" t="s">
         <v>19</v>
       </c>
@@ -1629,7 +1647,7 @@
         <v>19</v>
       </c>
       <c r="O24" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1640,7 +1658,7 @@
         <v>19</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>19</v>
@@ -1654,10 +1672,10 @@
       <c r="G25" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I25" s="1"/>
+      <c r="H25" s="1"/>
+      <c r="I25" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="J25" s="1" t="s">
         <v>19</v>
       </c>
@@ -1674,7 +1692,7 @@
         <v>19</v>
       </c>
       <c r="O25" s="1" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1684,7 +1702,9 @@
       <c r="B26" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C26" s="1"/>
+      <c r="C26" s="1" t="s">
+        <v>87</v>
+      </c>
       <c r="D26" s="1" t="s">
         <v>19</v>
       </c>
@@ -1700,10 +1720,10 @@
       <c r="H26" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I26" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J26" s="1"/>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="K26" s="1" t="s">
         <v>19</v>
       </c>
@@ -1717,7 +1737,50 @@
         <v>19</v>
       </c>
       <c r="O26" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="L27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="M27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="N27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1737,11 +1800,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="17.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="17.52"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1793,13 +1856,13 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>19</v>
@@ -1820,7 +1883,7 @@
         <v>19</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>23</v>
@@ -1835,19 +1898,19 @@
         <v>33</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="P2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>19</v>
@@ -1868,7 +1931,7 @@
         <v>19</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>38</v>
@@ -1883,19 +1946,19 @@
         <v>33</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="P3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>19</v>
@@ -1916,7 +1979,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>38</v>
@@ -1931,19 +1994,19 @@
         <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="P4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>19</v>
@@ -1964,7 +2027,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>23</v>
@@ -1979,7 +2042,7 @@
         <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="P5" s="1"/>
     </row>
@@ -2000,7 +2063,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O53"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.67"/>
@@ -2061,13 +2124,13 @@
         <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>19</v>
@@ -2082,7 +2145,7 @@
         <v>19</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J2" s="1" t="s">
         <v>19</v>
@@ -2100,7 +2163,7 @@
         <v>33</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2112,7 +2175,7 @@
         <v>17</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>19</v>
@@ -2127,7 +2190,7 @@
         <v>19</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>19</v>
@@ -2145,12 +2208,12 @@
         <v>33</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>32</v>
@@ -2159,7 +2222,7 @@
         <v>17</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>19</v>
@@ -2174,7 +2237,7 @@
         <v>19</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>19</v>
@@ -2192,7 +2255,7 @@
         <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2203,7 +2266,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>19</v>
@@ -2218,7 +2281,7 @@
         <v>19</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>19</v>
@@ -2236,7 +2299,7 @@
         <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2247,10 +2310,10 @@
         <v>16</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>19</v>
@@ -2283,7 +2346,7 @@
         <v>24</v>
       </c>
       <c r="O6" s="0" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2328,7 +2391,7 @@
         <v>24</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2342,13 +2405,13 @@
         <v>17</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>21</v>
@@ -2375,7 +2438,7 @@
         <v>24</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2397,16 +2460,16 @@
     </row>
     <row r="10" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>19</v>
@@ -2436,21 +2499,21 @@
         <v>24</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
     </row>
     <row r="11" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>19</v>
@@ -2480,27 +2543,27 @@
         <v>24</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>21</v>
@@ -2527,27 +2590,27 @@
         <v>24</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>19</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>21</v>
@@ -2574,21 +2637,21 @@
         <v>24</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>19</v>
@@ -2618,21 +2681,21 @@
         <v>24</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>19</v>
@@ -2662,21 +2725,21 @@
         <v>24</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>19</v>
@@ -2685,7 +2748,7 @@
         <v>1</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>19</v>
@@ -2709,21 +2772,21 @@
         <v>24</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>19</v>
@@ -2732,7 +2795,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>19</v>
@@ -2756,21 +2819,21 @@
         <v>24</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
     </row>
     <row r="18" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>19</v>
@@ -2800,21 +2863,21 @@
         <v>24</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
     </row>
     <row r="19" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E19" s="1" t="s">
         <v>19</v>
@@ -2844,21 +2907,21 @@
         <v>24</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>19</v>
@@ -2873,7 +2936,7 @@
         <v>19</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="J20" s="1" t="s">
         <v>19</v>
@@ -2891,21 +2954,21 @@
         <v>24</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>17</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>19</v>
@@ -2920,7 +2983,7 @@
         <v>19</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="J21" s="1" t="s">
         <v>19</v>
@@ -2938,7 +3001,7 @@
         <v>24</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3149,7 +3212,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O33"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.67"/>
@@ -3216,7 +3279,7 @@
         <v>17</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>19</v>
@@ -3249,18 +3312,18 @@
         <v>24</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>19</v>
@@ -3281,7 +3344,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>23</v>
@@ -3296,18 +3359,18 @@
         <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>19</v>
@@ -3328,7 +3391,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>38</v>
@@ -3343,18 +3406,18 @@
         <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>19</v>
@@ -3375,7 +3438,7 @@
         <v>19</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>23</v>
@@ -3390,18 +3453,18 @@
         <v>33</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>19</v>
@@ -3422,7 +3485,7 @@
         <v>19</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>38</v>
@@ -3437,18 +3500,18 @@
         <v>33</v>
       </c>
       <c r="O7" s="1" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>19</v>
@@ -3469,7 +3532,7 @@
         <v>19</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>23</v>
@@ -3484,18 +3547,18 @@
         <v>33</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>19</v>
@@ -3516,7 +3579,7 @@
         <v>19</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="K9" s="1" t="s">
         <v>23</v>
@@ -3531,18 +3594,18 @@
         <v>33</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="10" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>19</v>
@@ -3563,7 +3626,7 @@
         <v>19</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>38</v>
@@ -3578,18 +3641,18 @@
         <v>33</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>19</v>
@@ -3610,7 +3673,7 @@
         <v>19</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="K11" s="1" t="s">
         <v>38</v>
@@ -3625,18 +3688,18 @@
         <v>33</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
     </row>
     <row r="12" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>19</v>
@@ -3657,7 +3720,7 @@
         <v>19</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>23</v>
@@ -3672,18 +3735,18 @@
         <v>33</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>19</v>
@@ -3704,10 +3767,10 @@
         <v>19</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="L13" s="1" t="n">
         <v>10000003</v>
@@ -3719,18 +3782,18 @@
         <v>33</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>19</v>
@@ -3751,10 +3814,10 @@
         <v>19</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="L14" s="1" t="n">
         <v>10000003</v>
@@ -3766,18 +3829,18 @@
         <v>33</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="15" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>19</v>
@@ -3798,7 +3861,7 @@
         <v>19</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>23</v>
@@ -3813,18 +3876,18 @@
         <v>33</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>19</v>
@@ -3845,7 +3908,7 @@
         <v>19</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="K16" s="1" t="s">
         <v>38</v>
@@ -3860,18 +3923,18 @@
         <v>33</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>19</v>
@@ -3892,10 +3955,10 @@
         <v>19</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="L17" s="1" t="n">
         <v>10000003</v>
@@ -3907,42 +3970,42 @@
         <v>33</v>
       </c>
       <c r="O17" s="1" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K18" s="1" t="s">
         <v>138</v>
-      </c>
-      <c r="B18" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="K18" s="1" t="s">
-        <v>133</v>
       </c>
       <c r="L18" s="1" t="n">
         <v>10000003</v>
@@ -3954,18 +4017,18 @@
         <v>33</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>19</v>
@@ -3986,7 +4049,7 @@
         <v>19</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="K19" s="1" t="s">
         <v>38</v>
@@ -4001,18 +4064,18 @@
         <v>33</v>
       </c>
       <c r="O19" s="1" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
     </row>
     <row r="20" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>19</v>
@@ -4033,10 +4096,10 @@
         <v>19</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="L20" s="1" t="n">
         <v>10000003</v>
@@ -4048,18 +4111,18 @@
         <v>33</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="21" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>19</v>
@@ -4080,10 +4143,10 @@
         <v>19</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="L21" s="1" t="n">
         <v>10000003</v>
@@ -4095,18 +4158,18 @@
         <v>33</v>
       </c>
       <c r="O21" s="1" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
     </row>
     <row r="22" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>19</v>
@@ -4127,7 +4190,7 @@
         <v>19</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="K22" s="1" t="s">
         <v>23</v>
@@ -4142,7 +4205,7 @@
         <v>33</v>
       </c>
       <c r="O22" s="1" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4313,7 +4376,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:P25"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.67"/>
@@ -4374,10 +4437,10 @@
         <v>40</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>19</v>
@@ -4398,7 +4461,7 @@
         <v>19</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>23</v>
@@ -4413,7 +4476,7 @@
         <v>33</v>
       </c>
       <c r="O2" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="P2" s="1"/>
     </row>
@@ -4422,10 +4485,10 @@
         <v>40</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>19</v>
@@ -4446,7 +4509,7 @@
         <v>19</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>38</v>
@@ -4461,7 +4524,7 @@
         <v>33</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="P3" s="1"/>
     </row>
@@ -4470,10 +4533,10 @@
         <v>40</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>19</v>
@@ -4494,7 +4557,7 @@
         <v>19</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>38</v>
@@ -4509,7 +4572,7 @@
         <v>33</v>
       </c>
       <c r="O4" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="P4" s="1"/>
     </row>
@@ -4518,10 +4581,10 @@
         <v>40</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>19</v>
@@ -4542,7 +4605,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>23</v>
@@ -4557,7 +4620,7 @@
         <v>33</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="P5" s="1"/>
     </row>
@@ -4659,7 +4722,7 @@
         <v>40</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>42</v>
@@ -4704,7 +4767,7 @@
         <v>41</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>42</v>
@@ -4749,7 +4812,7 @@
         <v>41</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>42</v>

</xml_diff>